<commit_message>
refined code for perturbation based sensing
11/12/2025
</commit_message>
<xml_diff>
--- a/Raw Data/single force (10 trials)(perturbed)/Validation(1.5)(3tendon).xlsx
+++ b/Raw Data/single force (10 trials)(perturbed)/Validation(1.5)(3tendon).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://djpropertycom-my.sharepoint.com/personal/noah_familiajones_org/Documents/Work and Projects/Github/Whisker_Inspired_Sensing_CR/Raw Data/single force (10 trials)(perturbed)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4327" documentId="8_{DFFD6B0C-681F-42C8-B2E4-5D4B90AAE966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E053C78-8FF1-4563-A9E8-EE554E4686D8}"/>
+  <xr:revisionPtr revIDLastSave="4350" documentId="8_{DFFD6B0C-681F-42C8-B2E4-5D4B90AAE966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82CA90CF-99A7-466F-B68F-196908267B01}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="4" xr2:uid="{3D16C37F-3C74-4527-A308-796C339DFE9F}"/>
   </bookViews>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="42">
   <si>
     <t>Fx (N)</t>
   </si>
@@ -517,6 +517,9 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -527,9 +530,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1894,11 +1894,11 @@
       </c>
       <c r="R1" s="27"/>
       <c r="S1" s="27"/>
-      <c r="T1" s="34" t="s">
+      <c r="T1" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="U1" s="34"/>
-      <c r="V1" s="34"/>
+      <c r="U1" s="30"/>
+      <c r="V1" s="30"/>
       <c r="W1" s="28"/>
       <c r="X1" s="28"/>
       <c r="Y1" s="28"/>
@@ -2934,11 +2934,11 @@
       </c>
       <c r="R1" s="27"/>
       <c r="S1" s="27"/>
-      <c r="T1" s="34" t="s">
+      <c r="T1" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="U1" s="34"/>
-      <c r="V1" s="34"/>
+      <c r="U1" s="30"/>
+      <c r="V1" s="30"/>
       <c r="W1" s="28"/>
       <c r="X1" s="28"/>
       <c r="Y1" s="28"/>
@@ -3907,11 +3907,11 @@
       </c>
     </row>
     <row r="14" spans="1:25" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="30" t="s">
+      <c r="A14" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="31"/>
-      <c r="C14" s="32"/>
+      <c r="B14" s="32"/>
+      <c r="C14" s="33"/>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15">
@@ -5391,11 +5391,11 @@
       </c>
       <c r="R1" s="27"/>
       <c r="S1" s="27"/>
-      <c r="T1" s="34" t="s">
+      <c r="T1" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="U1" s="34"/>
-      <c r="V1" s="34"/>
+      <c r="U1" s="30"/>
+      <c r="V1" s="30"/>
       <c r="W1" s="28"/>
       <c r="X1" s="28"/>
       <c r="Y1" s="28"/>
@@ -6364,11 +6364,11 @@
       </c>
     </row>
     <row r="14" spans="1:25" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="30" t="s">
+      <c r="A14" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="31"/>
-      <c r="C14" s="32"/>
+      <c r="B14" s="32"/>
+      <c r="C14" s="33"/>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15">
@@ -7839,11 +7839,11 @@
       </c>
       <c r="R1" s="27"/>
       <c r="S1" s="27"/>
-      <c r="T1" s="34" t="s">
+      <c r="T1" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="U1" s="34"/>
-      <c r="V1" s="34"/>
+      <c r="U1" s="30"/>
+      <c r="V1" s="30"/>
       <c r="W1" s="28"/>
       <c r="X1" s="28"/>
       <c r="Y1" s="28"/>
@@ -8812,11 +8812,11 @@
       </c>
     </row>
     <row r="14" spans="1:25" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="30" t="s">
+      <c r="A14" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="31"/>
-      <c r="C14" s="32"/>
+      <c r="B14" s="32"/>
+      <c r="C14" s="33"/>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15">
@@ -10241,22 +10241,22 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="32"/>
-      <c r="H1" s="33" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="33"/>
+      <c r="H1" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
-      <c r="K1" s="31"/>
-      <c r="L1" s="31"/>
-      <c r="M1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="32"/>
+      <c r="L1" s="32"/>
+      <c r="M1" s="33"/>
     </row>
     <row r="2" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
@@ -16595,7 +16595,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="49" spans="26:37" x14ac:dyDescent="0.25">
+    <row r="49" spans="26:48" x14ac:dyDescent="0.25">
       <c r="Z49" t="s">
         <v>29</v>
       </c>
@@ -16629,8 +16629,32 @@
       <c r="AJ49" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="50" spans="26:37" x14ac:dyDescent="0.25">
+      <c r="AO49" t="s">
+        <v>29</v>
+      </c>
+      <c r="AP49">
+        <v>0.4</v>
+      </c>
+      <c r="AQ49">
+        <v>0.06</v>
+      </c>
+      <c r="AR49">
+        <v>1.5707963267948966</v>
+      </c>
+      <c r="AS49">
+        <v>0</v>
+      </c>
+      <c r="AT49">
+        <v>0</v>
+      </c>
+      <c r="AU49">
+        <v>0</v>
+      </c>
+      <c r="AV49" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="50" spans="26:48" x14ac:dyDescent="0.25">
       <c r="Z50" t="s">
         <v>29</v>
       </c>
@@ -16664,8 +16688,29 @@
       <c r="AJ50" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="51" spans="26:37" x14ac:dyDescent="0.25">
+      <c r="AP50">
+        <v>0.8</v>
+      </c>
+      <c r="AQ50">
+        <v>0.06</v>
+      </c>
+      <c r="AR50">
+        <v>1.5707963267948966</v>
+      </c>
+      <c r="AS50">
+        <v>0</v>
+      </c>
+      <c r="AT50">
+        <v>0</v>
+      </c>
+      <c r="AU50">
+        <v>0</v>
+      </c>
+      <c r="AV50" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="51" spans="26:48" x14ac:dyDescent="0.25">
       <c r="Z51" t="s">
         <v>29</v>
       </c>
@@ -16699,8 +16744,29 @@
       <c r="AJ51" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="52" spans="26:37" x14ac:dyDescent="0.25">
+      <c r="AP51">
+        <v>0.3</v>
+      </c>
+      <c r="AQ51">
+        <v>0.08</v>
+      </c>
+      <c r="AR51">
+        <v>1.5707963267948966</v>
+      </c>
+      <c r="AS51">
+        <v>0</v>
+      </c>
+      <c r="AT51">
+        <v>0</v>
+      </c>
+      <c r="AU51">
+        <v>0</v>
+      </c>
+      <c r="AV51" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="52" spans="26:48" x14ac:dyDescent="0.25">
       <c r="Z52" t="s">
         <v>29</v>
       </c>
@@ -16734,8 +16800,26 @@
       <c r="AJ52" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="53" spans="26:37" x14ac:dyDescent="0.25">
+      <c r="AP52">
+        <v>0.5</v>
+      </c>
+      <c r="AQ52">
+        <v>0.1</v>
+      </c>
+      <c r="AR52">
+        <v>1.5707963267948966</v>
+      </c>
+      <c r="AS52">
+        <v>0</v>
+      </c>
+      <c r="AT52">
+        <v>0</v>
+      </c>
+      <c r="AU52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="26:48" x14ac:dyDescent="0.25">
       <c r="Z53" t="s">
         <v>29</v>
       </c>
@@ -16769,8 +16853,29 @@
       <c r="AJ53" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="54" spans="26:37" x14ac:dyDescent="0.25">
+      <c r="AP53">
+        <v>0.7</v>
+      </c>
+      <c r="AQ53">
+        <v>0.1</v>
+      </c>
+      <c r="AR53">
+        <v>1.5707963267948966</v>
+      </c>
+      <c r="AS53">
+        <v>0</v>
+      </c>
+      <c r="AT53">
+        <v>0</v>
+      </c>
+      <c r="AU53">
+        <v>0</v>
+      </c>
+      <c r="AV53" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="54" spans="26:48" x14ac:dyDescent="0.25">
       <c r="Z54" t="s">
         <v>29</v>
       </c>
@@ -16804,8 +16909,29 @@
       <c r="AJ54" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="55" spans="26:37" x14ac:dyDescent="0.25">
+      <c r="AP54">
+        <v>0.4</v>
+      </c>
+      <c r="AQ54">
+        <v>0.16</v>
+      </c>
+      <c r="AR54">
+        <v>1.5707963267948966</v>
+      </c>
+      <c r="AS54">
+        <v>0</v>
+      </c>
+      <c r="AT54">
+        <v>0</v>
+      </c>
+      <c r="AU54">
+        <v>0</v>
+      </c>
+      <c r="AV54" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="55" spans="26:48" x14ac:dyDescent="0.25">
       <c r="Z55" t="s">
         <v>29</v>
       </c>
@@ -16839,8 +16965,29 @@
       <c r="AJ55" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="56" spans="26:37" x14ac:dyDescent="0.25">
+      <c r="AP55">
+        <v>0.6</v>
+      </c>
+      <c r="AQ55">
+        <v>0.16</v>
+      </c>
+      <c r="AR55">
+        <v>1.5707963267948966</v>
+      </c>
+      <c r="AS55">
+        <v>0</v>
+      </c>
+      <c r="AT55">
+        <v>0</v>
+      </c>
+      <c r="AU55">
+        <v>0</v>
+      </c>
+      <c r="AV55" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="56" spans="26:48" x14ac:dyDescent="0.25">
       <c r="Z56" t="s">
         <v>29</v>
       </c>
@@ -16876,6 +17023,73 @@
       </c>
       <c r="AK56" t="s">
         <v>38</v>
+      </c>
+      <c r="AP56">
+        <v>0.8</v>
+      </c>
+      <c r="AQ56">
+        <v>0.18</v>
+      </c>
+      <c r="AR56">
+        <v>1.5707963267948966</v>
+      </c>
+      <c r="AS56">
+        <v>0</v>
+      </c>
+      <c r="AT56">
+        <v>0</v>
+      </c>
+      <c r="AU56">
+        <v>0</v>
+      </c>
+      <c r="AV56" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="57" spans="26:48" x14ac:dyDescent="0.25">
+      <c r="AP57">
+        <v>0.3</v>
+      </c>
+      <c r="AQ57">
+        <v>0.2</v>
+      </c>
+      <c r="AR57">
+        <v>1.5707963267948966</v>
+      </c>
+      <c r="AS57">
+        <v>0</v>
+      </c>
+      <c r="AT57">
+        <v>0</v>
+      </c>
+      <c r="AU57">
+        <v>0</v>
+      </c>
+      <c r="AV57" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="58" spans="26:48" x14ac:dyDescent="0.25">
+      <c r="AP58">
+        <v>0.7</v>
+      </c>
+      <c r="AQ58">
+        <v>0.2</v>
+      </c>
+      <c r="AR58">
+        <v>1.5707963267948966</v>
+      </c>
+      <c r="AS58">
+        <v>0</v>
+      </c>
+      <c r="AT58">
+        <v>0</v>
+      </c>
+      <c r="AU58">
+        <v>0</v>
+      </c>
+      <c r="AV58" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
@@ -17398,16 +17612,16 @@
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE208467-E14A-4CB9-9FC8-72DFB8E94FF2}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="08a9f8ec-165a-4165-a8e9-ed45c2de7bcb"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="08a9f8ec-165a-4165-a8e9-ed45c2de7bcb"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>